<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-29 14:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001524 - ATACAMA KOZAN.xlsx
+++ b/data/50001524 - ATACAMA KOZAN.xlsx
@@ -3834,7 +3834,7 @@
         <v>46114.76051153935</v>
       </c>
       <c r="D42" s="5">
-        <v>46114.76064238426</v>
+        <v>46202.187087708335</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>154</v>
@@ -3872,8 +3872,8 @@
       <c r="P42" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="Q42" s="11" t="s">
-        <v>106</v>
+      <c r="Q42" s="12" t="s">
+        <v>56</v>
       </c>
       <c r="R42" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-23 13:43 UTC
</commit_message>
<xml_diff>
--- a/data/50001524 - ATACAMA KOZAN.xlsx
+++ b/data/50001524 - ATACAMA KOZAN.xlsx
@@ -409,154 +409,154 @@
     <t>Generación OC motor,Fabricación motor,Planos motor proveedor</t>
   </si>
   <si>
+    <t>1213470416901260</t>
+  </si>
+  <si>
+    <t>Generación OC motor</t>
+  </si>
+  <si>
+    <t>Fabricación motor,Planos motor proveedor,Motor</t>
+  </si>
+  <si>
+    <t>1213470416901261</t>
+  </si>
+  <si>
+    <t>Fabricación motor</t>
+  </si>
+  <si>
+    <t>Motor,Recepcion  motor</t>
+  </si>
+  <si>
+    <t>1213470416901262</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>Motor,Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213470416901263</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>1213470416901264</t>
+  </si>
+  <si>
+    <t>Generación OC materiales</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>1213470416901265</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Materiales a codigo // compras locales aprovisionamientomiento:,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213470416901266</t>
+  </si>
+  <si>
+    <t>Sensores</t>
+  </si>
+  <si>
+    <t>Generación Oc sensores,Fabricación Sensores</t>
+  </si>
+  <si>
+    <t>1213470416901267</t>
+  </si>
+  <si>
+    <t>Generación Oc sensores</t>
+  </si>
+  <si>
+    <t>Fabricación Sensores,Sensores</t>
+  </si>
+  <si>
+    <t>1213470416901268</t>
+  </si>
+  <si>
+    <t>Fabricación Sensores</t>
+  </si>
+  <si>
+    <t>Sensores,Recepcion sensores</t>
+  </si>
+  <si>
+    <t>1213470416901269</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>Planos Preliminar,Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213470416901270</t>
+  </si>
+  <si>
+    <t>Planos Preliminar</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t>Planos Definitivos,Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>1213470416901271</t>
+  </si>
+  <si>
+    <t>Planos Definitivos</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor,Planos Preliminar</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:,Check planos</t>
+  </si>
+  <si>
+    <t>1213561126963324</t>
+  </si>
+  <si>
+    <t>Check planos</t>
+  </si>
+  <si>
+    <t>Armado,Control de calidad Armado,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor</t>
+  </si>
+  <si>
+    <t>1213561126963325</t>
+  </si>
+  <si>
+    <t>Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>Pruebas FAT</t>
+  </si>
+  <si>
+    <t>RE-PINTADO</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213470416901260</t>
-  </si>
-  <si>
-    <t>Generación OC motor</t>
-  </si>
-  <si>
-    <t>Fabricación motor,Planos motor proveedor,Motor</t>
-  </si>
-  <si>
-    <t>1213470416901261</t>
-  </si>
-  <si>
-    <t>Fabricación motor</t>
-  </si>
-  <si>
-    <t>Motor,Recepcion  motor</t>
-  </si>
-  <si>
-    <t>1213470416901262</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>Motor,Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213470416901263</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>1213470416901264</t>
-  </si>
-  <si>
-    <t>Generación OC materiales</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>1213470416901265</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Materiales a codigo // compras locales aprovisionamientomiento:,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213470416901266</t>
-  </si>
-  <si>
-    <t>Sensores</t>
-  </si>
-  <si>
-    <t>Generación Oc sensores,Fabricación Sensores</t>
-  </si>
-  <si>
-    <t>1213470416901267</t>
-  </si>
-  <si>
-    <t>Generación Oc sensores</t>
-  </si>
-  <si>
-    <t>Fabricación Sensores,Sensores</t>
-  </si>
-  <si>
-    <t>1213470416901268</t>
-  </si>
-  <si>
-    <t>Fabricación Sensores</t>
-  </si>
-  <si>
-    <t>Sensores,Recepcion sensores</t>
-  </si>
-  <si>
-    <t>1213470416901269</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>Planos Preliminar,Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213470416901270</t>
-  </si>
-  <si>
-    <t>Planos Preliminar</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t>Planos Definitivos,Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>1213470416901271</t>
-  </si>
-  <si>
-    <t>Planos Definitivos</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor,Planos Preliminar</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:,Check planos</t>
-  </si>
-  <si>
-    <t>1213561126963324</t>
-  </si>
-  <si>
-    <t>Check planos</t>
-  </si>
-  <si>
-    <t>Armado,Control de calidad Armado,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor</t>
-  </si>
-  <si>
-    <t>1213561126963325</t>
-  </si>
-  <si>
-    <t>Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>Pruebas FAT</t>
-  </si>
-  <si>
-    <t>RE-PINTADO</t>
   </si>
   <si>
     <t>1213470416901272</t>
@@ -3396,7 +3396,7 @@
         <v>46114.76327634259</v>
       </c>
       <c r="D35" s="8">
-        <v>46218.1834093287</v>
+        <v>46226.18144005787</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>130</v>
@@ -3434,8 +3434,8 @@
       <c r="P35" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="Q35" s="12" t="s">
-        <v>132</v>
+      <c r="Q35" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="R35" s="9">
         <v>1</v>
@@ -3452,7 +3452,7 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B36" s="5">
         <v>46080.77828773148</v>
@@ -3464,7 +3464,7 @@
         <v>46114.76319354167</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
@@ -3497,7 +3497,7 @@
         <v>77</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Q36" s="11" t="s">
         <v>107</v>
@@ -3513,7 +3513,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B37" s="8">
         <v>46080.77828799769</v>
@@ -3525,7 +3525,7 @@
         <v>46114.763248877316</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
@@ -3555,10 +3555,10 @@
         <v>130</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q37" s="11" t="s">
         <v>107</v>
@@ -3574,7 +3574,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B38" s="5">
         <v>46080.77828825232</v>
@@ -3586,7 +3586,7 @@
         <v>46114.7632599537</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
@@ -3616,10 +3616,10 @@
         <v>130</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q38" s="11" t="s">
         <v>107</v>
@@ -3635,7 +3635,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B39" s="8">
         <v>46080.778288518515</v>
@@ -3647,16 +3647,16 @@
         <v>46149.197581886576</v>
       </c>
       <c r="E39" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="F39" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="9" t="s">
+      <c r="H39" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>145</v>
       </c>
       <c r="I39" s="8">
         <v>46100</v>
@@ -3677,7 +3677,7 @@
         <v>97</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>97</v>
@@ -3700,7 +3700,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B40" s="5">
         <v>46080.77828673611</v>
@@ -3712,16 +3712,16 @@
         <v>46121.8600697338</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="I40" s="5">
         <v>46100</v>
@@ -3739,13 +3739,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q40" s="11" t="s">
         <v>107</v>
@@ -3761,7 +3761,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B41" s="8">
         <v>46080.77828702546</v>
@@ -3773,16 +3773,16 @@
         <v>46121.86006597222</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H41" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>145</v>
       </c>
       <c r="I41" s="8">
         <v>46120</v>
@@ -3800,13 +3800,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O41" s="9" t="s">
         <v>94</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q41" s="11" t="s">
         <v>107</v>
@@ -3822,7 +3822,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B42" s="5">
         <v>46080.77828724537</v>
@@ -3834,16 +3834,16 @@
         <v>46210.17465634259</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="H42" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="I42" s="5">
         <v>46100</v>
@@ -3864,7 +3864,7 @@
         <v>97</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>97</v>
@@ -3887,7 +3887,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B43" s="8">
         <v>46080.77828748843</v>
@@ -3899,16 +3899,16 @@
         <v>46114.76045094908</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H43" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>145</v>
       </c>
       <c r="I43" s="8">
         <v>46100</v>
@@ -3926,13 +3926,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O43" s="9" t="s">
         <v>91</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Q43" s="11" t="s">
         <v>107</v>
@@ -3948,7 +3948,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B44" s="5">
         <v>46080.77828770834</v>
@@ -3960,16 +3960,16 @@
         <v>46114.7604978125</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="I44" s="5">
         <v>46129</v>
@@ -3987,13 +3987,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q44" s="11" t="s">
         <v>107</v>
@@ -4009,7 +4009,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B45" s="8">
         <v>46080.778287939815</v>
@@ -4021,7 +4021,7 @@
         <v>46141.772341724536</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>25</v>
@@ -4045,7 +4045,7 @@
         <v>26</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P45" s="9" t="s">
         <v>26</v>
@@ -4058,7 +4058,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B46" s="5">
         <v>46080.778288182875</v>
@@ -4070,16 +4070,16 @@
         <v>46127.67810105324</v>
       </c>
       <c r="E46" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G46" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="F46" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G46" s="6" t="s">
+      <c r="H46" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>167</v>
       </c>
       <c r="I46" s="5">
         <v>46098</v>
@@ -4097,13 +4097,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>67</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q46" s="10" t="s">
         <v>31</v>
@@ -4123,7 +4123,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B47" s="8">
         <v>46080.77828842592</v>
@@ -4135,16 +4135,16 @@
         <v>46158.16995894676</v>
       </c>
       <c r="E47" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" s="9" t="s">
+      <c r="H47" s="9" t="s">
         <v>171</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>172</v>
       </c>
       <c r="I47" s="8">
         <v>46140</v>
@@ -4162,13 +4162,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O47" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="P47" s="9" t="s">
         <v>173</v>
-      </c>
-      <c r="P47" s="9" t="s">
-        <v>174</v>
       </c>
       <c r="Q47" s="10" t="s">
         <v>31</v>
@@ -4188,7 +4188,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B48" s="5">
         <v>46087.53644159722</v>
@@ -4200,16 +4200,16 @@
         <v>46161.20788581019</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>171</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>172</v>
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="5">
@@ -4225,13 +4225,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q48" s="10" t="s">
         <v>31</v>
@@ -4251,7 +4251,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B49" s="8">
         <v>46087.536521331014</v>
@@ -4260,19 +4260,19 @@
         <v>46140.83887265046</v>
       </c>
       <c r="D49" s="8">
-        <v>46141.771787060185</v>
+        <v>46226.177547245374</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="H49" s="9" t="s">
         <v>166</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>167</v>
       </c>
       <c r="I49" s="8">
         <v>46233</v>
@@ -4290,16 +4290,16 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O49" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="P49" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="P49" s="9" t="s">
+      <c r="Q49" s="12" t="s">
         <v>181</v>
-      </c>
-      <c r="Q49" s="11" t="s">
-        <v>107</v>
       </c>
       <c r="R49" s="9">
         <v>1</v>
@@ -4407,7 +4407,7 @@
         <v>183</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P51" s="9" t="s">
         <v>189</v>
@@ -4960,13 +4960,13 @@
         <v>183</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>221</v>
       </c>
       <c r="Q60" s="12" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="R60" s="6">
         <v>1</v>
@@ -5025,7 +5025,7 @@
         <v>183</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>224</v>
@@ -5275,7 +5275,7 @@
         <v>236</v>
       </c>
       <c r="Q65" s="12" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="R65" s="9">
         <v>1</v>
@@ -5499,7 +5499,7 @@
         <v>46225.18881381945</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>26</v>
@@ -5535,7 +5535,7 @@
         <v>248</v>
       </c>
       <c r="Q69" s="12" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="R69" s="9">
         <v>1</v>
@@ -5564,7 +5564,7 @@
         <v>46223.80689234954</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5594,7 +5594,7 @@
         <v>228</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>250</v>
@@ -5708,7 +5708,7 @@
         <v>252</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>258</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-31 15:28 UTC
</commit_message>
<xml_diff>
--- a/data/50001524 - ATACAMA KOZAN.xlsx
+++ b/data/50001524 - ATACAMA KOZAN.xlsx
@@ -556,214 +556,214 @@
     <t>RE-PINTADO</t>
   </si>
   <si>
+    <t>1213470416901272</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213470416901273</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
+  </si>
+  <si>
+    <t>1213470416901274</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>Bodega:,Preparación Materiales</t>
+  </si>
+  <si>
+    <t>1213470416901275</t>
+  </si>
+  <si>
+    <t>Caldereria:</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,Armado,Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1213470416901276</t>
+  </si>
+  <si>
+    <t>Preparación Materiales</t>
+  </si>
+  <si>
+    <t>Nicolás Mol</t>
+  </si>
+  <si>
+    <t>nicolas.mol@zitron.com</t>
+  </si>
+  <si>
+    <t>Armado,Caldereria:</t>
+  </si>
+  <si>
+    <t>1213470416901277</t>
+  </si>
+  <si>
+    <t>Armado</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,Check planos</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado,Caldereria:</t>
+  </si>
+  <si>
+    <t>1213470416901278</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>Armado,Check planos</t>
+  </si>
+  <si>
+    <t>Caldereria:,Revestimiento</t>
+  </si>
+  <si>
+    <t>1213470416901279</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete,Recepcion Alabe,Recepcion  motor,Recepcion sensores,Recepcion Tableros</t>
+  </si>
+  <si>
+    <t>1213470416901280</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Rodete</t>
+  </si>
+  <si>
+    <t>1213470416901281</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Alabe</t>
+  </si>
+  <si>
+    <t>1213470416901282</t>
+  </si>
+  <si>
+    <t>Recepcion  motor</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje motor</t>
+  </si>
+  <si>
+    <t>1213470416901283</t>
+  </si>
+  <si>
+    <t>Recepcion sensores</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Sensor</t>
+  </si>
+  <si>
+    <t>1213458788103573</t>
+  </si>
+  <si>
+    <t>Bodega:,Revision Tableros</t>
+  </si>
+  <si>
+    <t>1213470416901284</t>
+  </si>
+  <si>
+    <t>Montaje:</t>
+  </si>
+  <si>
+    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor,RE-PINTADO,Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213470416901285</t>
+  </si>
+  <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor,Montaje:</t>
+  </si>
+  <si>
+    <t>1213470416901286</t>
+  </si>
+  <si>
+    <t>Montaje motor</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion  motor,Check planos</t>
+  </si>
+  <si>
+    <t>Montaje:,Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213470416901287</t>
+  </si>
+  <si>
+    <t>Montaje Alabe</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion Alabe,Check planos</t>
+  </si>
+  <si>
+    <t>1213470416901288</t>
+  </si>
+  <si>
+    <t>Montaje Rodete</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion Rodete,Check planos</t>
+  </si>
+  <si>
+    <t>1213470416901289</t>
+  </si>
+  <si>
+    <t>Montaje Sensor</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion sensores,Check planos</t>
+  </si>
+  <si>
+    <t>1213470416901290</t>
+  </si>
+  <si>
+    <t>Montaje Sensor,Montaje motor,Montaje Alabe,Montaje Rodete</t>
+  </si>
+  <si>
+    <t>Montaje:,Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213470414925601</t>
+  </si>
+  <si>
+    <t>Montaje:,Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213470416901272</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213470416901273</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
-  </si>
-  <si>
-    <t>1213470416901274</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>Bodega:,Preparación Materiales</t>
-  </si>
-  <si>
-    <t>1213470416901275</t>
-  </si>
-  <si>
-    <t>Caldereria:</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Armado,Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1213470416901276</t>
-  </si>
-  <si>
-    <t>Preparación Materiales</t>
-  </si>
-  <si>
-    <t>Nicolás Mol</t>
-  </si>
-  <si>
-    <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>Armado,Caldereria:</t>
-  </si>
-  <si>
-    <t>1213470416901277</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Check planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado,Caldereria:</t>
-  </si>
-  <si>
-    <t>1213470416901278</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>Armado,Check planos</t>
-  </si>
-  <si>
-    <t>Caldereria:,Revestimiento</t>
-  </si>
-  <si>
-    <t>1213470416901279</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete,Recepcion Alabe,Recepcion  motor,Recepcion sensores,Recepcion Tableros</t>
-  </si>
-  <si>
-    <t>1213470416901280</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Rodete</t>
-  </si>
-  <si>
-    <t>1213470416901281</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Alabe</t>
-  </si>
-  <si>
-    <t>1213470416901282</t>
-  </si>
-  <si>
-    <t>Recepcion  motor</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje motor</t>
-  </si>
-  <si>
-    <t>1213470416901283</t>
-  </si>
-  <si>
-    <t>Recepcion sensores</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Sensor</t>
-  </si>
-  <si>
-    <t>1213458788103573</t>
-  </si>
-  <si>
-    <t>Bodega:,Revision Tableros</t>
-  </si>
-  <si>
-    <t>1213470416901284</t>
-  </si>
-  <si>
-    <t>Montaje:</t>
-  </si>
-  <si>
-    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor,RE-PINTADO,Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213470416901285</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor,Montaje:</t>
-  </si>
-  <si>
-    <t>1213470416901286</t>
-  </si>
-  <si>
-    <t>Montaje motor</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion  motor,Check planos</t>
-  </si>
-  <si>
-    <t>Montaje:,Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213470416901287</t>
-  </si>
-  <si>
-    <t>Montaje Alabe</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion Alabe,Check planos</t>
-  </si>
-  <si>
-    <t>1213470416901288</t>
-  </si>
-  <si>
-    <t>Montaje Rodete</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion Rodete,Check planos</t>
-  </si>
-  <si>
-    <t>1213470416901289</t>
-  </si>
-  <si>
-    <t>Montaje Sensor</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion sensores,Check planos</t>
-  </si>
-  <si>
-    <t>1213470416901290</t>
-  </si>
-  <si>
-    <t>Montaje Sensor,Montaje motor,Montaje Alabe,Montaje Rodete</t>
-  </si>
-  <si>
-    <t>Montaje:,Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213470414925601</t>
-  </si>
-  <si>
-    <t>Montaje:,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
     <t>1213470414925602</t>
@@ -4260,7 +4260,7 @@
         <v>46140.83887265046</v>
       </c>
       <c r="D49" s="8">
-        <v>46226.177547245374</v>
+        <v>46234.1840334375</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4298,8 +4298,8 @@
       <c r="P49" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="Q49" s="12" t="s">
-        <v>181</v>
+      <c r="Q49" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="R49" s="9">
         <v>1</v>
@@ -4316,7 +4316,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B50" s="5">
         <v>46080.77828866898</v>
@@ -4328,7 +4328,7 @@
         <v>46141.772585231476</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>25</v>
@@ -4352,7 +4352,7 @@
         <v>26</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4365,7 +4365,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B51" s="8">
         <v>46080.77828892361</v>
@@ -4377,16 +4377,16 @@
         <v>46151.18472762732</v>
       </c>
       <c r="E51" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G51" s="9" t="s">
+      <c r="H51" s="9" t="s">
         <v>187</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>188</v>
       </c>
       <c r="I51" s="8">
         <v>46149</v>
@@ -4404,13 +4404,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O51" s="9" t="s">
         <v>148</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="Q51" s="10" t="s">
         <v>31</v>
@@ -4430,7 +4430,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B52" s="5">
         <v>46080.77828760417</v>
@@ -4442,16 +4442,16 @@
         <v>46155.20414789351</v>
       </c>
       <c r="E52" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G52" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>192</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>193</v>
       </c>
       <c r="I52" s="5">
         <v>46153</v>
@@ -4469,13 +4469,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="Q52" s="10" t="s">
         <v>31</v>
@@ -4495,7 +4495,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B53" s="8">
         <v>46080.778288009256</v>
@@ -4507,7 +4507,7 @@
         <v>46141.77186175926</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>25</v>
@@ -4531,7 +4531,7 @@
         <v>26</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P53" s="9" t="s">
         <v>26</v>
@@ -4544,7 +4544,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B54" s="5">
         <v>46080.77828832176</v>
@@ -4556,16 +4556,16 @@
         <v>46165.18131118055</v>
       </c>
       <c r="E54" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="F54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G54" s="6" t="s">
+      <c r="H54" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="I54" s="5">
         <v>46155</v>
@@ -4583,13 +4583,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Q54" s="10" t="s">
         <v>31</v>
@@ -4609,7 +4609,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B55" s="8">
         <v>46080.77828861111</v>
@@ -4621,16 +4621,16 @@
         <v>46170.185211909724</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="H55" s="9" t="s">
         <v>200</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>201</v>
       </c>
       <c r="I55" s="8">
         <v>46167</v>
@@ -4648,13 +4648,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O55" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="P55" s="9" t="s">
         <v>205</v>
-      </c>
-      <c r="P55" s="9" t="s">
-        <v>206</v>
       </c>
       <c r="Q55" s="10" t="s">
         <v>31</v>
@@ -4674,7 +4674,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B56" s="5">
         <v>46080.778288912035</v>
@@ -4686,16 +4686,16 @@
         <v>46172.2027446875</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>192</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>193</v>
       </c>
       <c r="I56" s="5">
         <v>46170</v>
@@ -4713,13 +4713,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O56" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="P56" s="6" t="s">
         <v>209</v>
-      </c>
-      <c r="P56" s="6" t="s">
-        <v>210</v>
       </c>
       <c r="Q56" s="10" t="s">
         <v>31</v>
@@ -4739,7 +4739,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B57" s="8">
         <v>46080.77828921296</v>
@@ -4751,7 +4751,7 @@
         <v>46141.77231675926</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>25</v>
@@ -4775,7 +4775,7 @@
         <v>26</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="P57" s="9" t="s">
         <v>26</v>
@@ -4788,7 +4788,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B58" s="5">
         <v>46080.77828957176</v>
@@ -4800,16 +4800,16 @@
         <v>46156.16908381945</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="I58" s="5">
         <v>46154</v>
@@ -4827,13 +4827,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>127</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Q58" s="10" t="s">
         <v>31</v>
@@ -4853,7 +4853,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B59" s="8">
         <v>46080.77828986111</v>
@@ -4865,16 +4865,16 @@
         <v>46218.18543643519</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="H59" s="9" t="s">
         <v>187</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>188</v>
       </c>
       <c r="I59" s="8">
         <v>46216</v>
@@ -4892,13 +4892,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O59" s="9" t="s">
         <v>127</v>
       </c>
       <c r="P59" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="Q59" s="10" t="s">
         <v>31</v>
@@ -4918,7 +4918,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B60" s="5">
         <v>46080.778290138885</v>
@@ -4930,16 +4930,16 @@
         <v>46228.20468340278</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="I60" s="5">
         <v>46226</v>
@@ -4957,13 +4957,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>136</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Q60" s="10" t="s">
         <v>31</v>
@@ -4983,7 +4983,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B61" s="8">
         <v>46080.778290393515</v>
@@ -4995,16 +4995,16 @@
         <v>46212.18789364584</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="H61" s="9" t="s">
         <v>187</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>188</v>
       </c>
       <c r="I61" s="8">
         <v>46210</v>
@@ -5022,13 +5022,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O61" s="9" t="s">
         <v>158</v>
       </c>
       <c r="P61" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q61" s="10" t="s">
         <v>31</v>
@@ -5048,7 +5048,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B62" s="5">
         <v>46080.7854796875</v>
@@ -5066,10 +5066,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="I62" s="5">
         <v>46199</v>
@@ -5087,13 +5087,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>118</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="Q62" s="10" t="s">
         <v>31</v>
@@ -5113,7 +5113,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B63" s="8">
         <v>46080.77828662037</v>
@@ -5125,7 +5125,7 @@
         <v>46141.71127789352</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>25</v>
@@ -5149,7 +5149,7 @@
         <v>26</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="P63" s="9" t="s">
         <v>26</v>
@@ -5162,7 +5162,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B64" s="5">
         <v>46080.77828694445</v>
@@ -5174,7 +5174,7 @@
         <v>46223.80691788194</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
@@ -5201,13 +5201,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="Q64" s="10" t="s">
         <v>31</v>
@@ -5227,7 +5227,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B65" s="8">
         <v>46080.778287187495</v>
@@ -5239,7 +5239,7 @@
         <v>46232.187510625</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
@@ -5266,13 +5266,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O65" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="P65" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="P65" s="9" t="s">
-        <v>236</v>
       </c>
       <c r="Q65" s="10" t="s">
         <v>31</v>
@@ -5292,7 +5292,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B66" s="5">
         <v>46080.77828746528</v>
@@ -5304,7 +5304,7 @@
         <v>46223.80691021991</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
@@ -5331,13 +5331,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Q66" s="10" t="s">
         <v>31</v>
@@ -5357,7 +5357,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B67" s="8">
         <v>46080.77828770834</v>
@@ -5369,7 +5369,7 @@
         <v>46224.20544344907</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
@@ -5396,13 +5396,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Q67" s="10" t="s">
         <v>31</v>
@@ -5422,7 +5422,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B68" s="5">
         <v>46080.77828796297</v>
@@ -5434,7 +5434,7 @@
         <v>46223.80690207176</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
@@ -5461,13 +5461,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Q68" s="10" t="s">
         <v>31</v>
@@ -5487,7 +5487,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B69" s="8">
         <v>46080.778288217596</v>
@@ -5526,13 +5526,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O69" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="P69" s="9" t="s">
         <v>247</v>
-      </c>
-      <c r="P69" s="9" t="s">
-        <v>248</v>
       </c>
       <c r="Q69" s="10" t="s">
         <v>31</v>
@@ -5552,7 +5552,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B70" s="5">
         <v>46080.77828846065</v>
@@ -5591,16 +5591,16 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>178</v>
       </c>
       <c r="P70" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q70" s="12" t="s">
         <v>250</v>
-      </c>
-      <c r="Q70" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="R70" s="6">
         <v>1</v>
@@ -5714,7 +5714,7 @@
         <v>258</v>
       </c>
       <c r="Q72" s="12" t="s">
-        <v>181</v>
+        <v>250</v>
       </c>
       <c r="R72" s="6">
         <v>1</v>
@@ -5779,7 +5779,7 @@
         <v>262</v>
       </c>
       <c r="Q73" s="12" t="s">
-        <v>181</v>
+        <v>250</v>
       </c>
       <c r="R73" s="9">
         <v>1</v>
@@ -5814,10 +5814,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="I74" s="5">
         <v>46239</v>
@@ -5844,7 +5844,7 @@
         <v>265</v>
       </c>
       <c r="Q74" s="12" t="s">
-        <v>181</v>
+        <v>250</v>
       </c>
       <c r="R74" s="6">
         <v>1</v>
@@ -5879,10 +5879,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="H75" s="9" t="s">
         <v>200</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>201</v>
       </c>
       <c r="I75" s="8">
         <v>46240</v>
@@ -5909,7 +5909,7 @@
         <v>268</v>
       </c>
       <c r="Q75" s="12" t="s">
-        <v>181</v>
+        <v>250</v>
       </c>
       <c r="R75" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-01 10:37 Chile
</commit_message>
<xml_diff>
--- a/data/50001524 - ATACAMA KOZAN.xlsx
+++ b/data/50001524 - ATACAMA KOZAN.xlsx
@@ -763,31 +763,31 @@
     <t>Montaje:,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
+    <t>1213470414925602</t>
+  </si>
+  <si>
+    <t>Logistica:</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
+  </si>
+  <si>
+    <t>1213470414925603</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>Karin Pinto</t>
+  </si>
+  <si>
+    <t>kpinto@zitron.com</t>
+  </si>
+  <si>
+    <t>Embalaje,Logistica:</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213470414925602</t>
-  </si>
-  <si>
-    <t>Logistica:</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
-  </si>
-  <si>
-    <t>1213470414925603</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente</t>
-  </si>
-  <si>
-    <t>Karin Pinto</t>
-  </si>
-  <si>
-    <t>kpinto@zitron.com</t>
-  </si>
-  <si>
-    <t>Embalaje,Logistica:</t>
   </si>
   <si>
     <t>1213470414925604</t>
@@ -5561,7 +5561,7 @@
         <v>46140.8390024074</v>
       </c>
       <c r="D70" s="5">
-        <v>46227.19814736111</v>
+        <v>46235.19700590278</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>180</v>
@@ -5599,8 +5599,8 @@
       <c r="P70" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="Q70" s="12" t="s">
-        <v>250</v>
+      <c r="Q70" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="R70" s="6">
         <v>1</v>
@@ -5617,7 +5617,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B71" s="8">
         <v>46080.7782887037</v>
@@ -5629,7 +5629,7 @@
         <v>46141.712052731484</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>25</v>
@@ -5653,7 +5653,7 @@
         <v>26</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="P71" s="9" t="s">
         <v>26</v>
@@ -5666,7 +5666,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B72" s="5">
         <v>46080.77828895833</v>
@@ -5678,16 +5678,16 @@
         <v>46230.16861260417</v>
       </c>
       <c r="E72" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G72" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="F72" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G72" s="6" t="s">
+      <c r="H72" s="6" t="s">
         <v>256</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>257</v>
       </c>
       <c r="I72" s="5">
         <v>46237</v>
@@ -5705,16 +5705,16 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>180</v>
       </c>
       <c r="P72" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q72" s="12" t="s">
         <v>258</v>
-      </c>
-      <c r="Q72" s="12" t="s">
-        <v>250</v>
       </c>
       <c r="R72" s="6">
         <v>1</v>
@@ -5770,7 +5770,7 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O73" s="9" t="s">
         <v>261</v>
@@ -5779,7 +5779,7 @@
         <v>262</v>
       </c>
       <c r="Q73" s="12" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="R73" s="9">
         <v>1</v>
@@ -5835,7 +5835,7 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>260</v>
@@ -5844,7 +5844,7 @@
         <v>265</v>
       </c>
       <c r="Q74" s="12" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="R74" s="6">
         <v>1</v>
@@ -5900,7 +5900,7 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O75" s="9" t="s">
         <v>264</v>
@@ -5909,7 +5909,7 @@
         <v>268</v>
       </c>
       <c r="Q75" s="12" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="R75" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-07 01:04 UTC
</commit_message>
<xml_diff>
--- a/data/50001524 - ATACAMA KOZAN.xlsx
+++ b/data/50001524 - ATACAMA KOZAN.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="278">
   <si>
     <t>50001524 - ATACAMA KOZAN</t>
   </si>
@@ -5907,9 +5907,11 @@
       <c r="B76" s="5">
         <v>46080.77828809028</v>
       </c>
-      <c r="C76" s="6"/>
+      <c r="C76" s="5">
+        <v>46240.815848865735</v>
+      </c>
       <c r="D76" s="5">
-        <v>46090.61092975695</v>
+        <v>46240.815850011575</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>270</v>
@@ -5942,8 +5944,12 @@
         <v>26</v>
       </c>
       <c r="Q76" s="6"/>
-      <c r="R76" s="6"/>
-      <c r="S76" s="6"/>
+      <c r="R76" s="6">
+        <v>1</v>
+      </c>
+      <c r="S76" s="11" t="s">
+        <v>32</v>
+      </c>
       <c r="T76" s="6"/>
       <c r="U76" s="6"/>
     </row>
@@ -5954,9 +5960,11 @@
       <c r="B77" s="8">
         <v>46080.77828868055</v>
       </c>
-      <c r="C77" s="9"/>
+      <c r="C77" s="8">
+        <v>46240.815745381944</v>
+      </c>
       <c r="D77" s="8">
-        <v>46141.711969386575</v>
+        <v>46240.81576049769</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>72</v>
@@ -5998,10 +6006,10 @@
         <v>107</v>
       </c>
       <c r="R77" s="9">
-        <v>0</v>
-      </c>
-      <c r="S77" s="10" t="s">
-        <v>108</v>
+        <v>1</v>
+      </c>
+      <c r="S77" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="T77" s="8">
         <v>46241</v>
@@ -6017,9 +6025,11 @@
       <c r="B78" s="5">
         <v>46080.77828835648</v>
       </c>
-      <c r="C78" s="6"/>
+      <c r="C78" s="5">
+        <v>46240.81575891204</v>
+      </c>
       <c r="D78" s="5">
-        <v>46141.711970648146</v>
+        <v>46240.81577349537</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>277</v>
@@ -6061,10 +6071,10 @@
         <v>107</v>
       </c>
       <c r="R78" s="6">
-        <v>0</v>
-      </c>
-      <c r="S78" s="10" t="s">
-        <v>108</v>
+        <v>1</v>
+      </c>
+      <c r="S78" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="T78" s="5">
         <v>46241</v>

</xml_diff>